<commit_message>
Update ANTAM gold prices
</commit_message>
<xml_diff>
--- a/data/harga_emas_antam.xlsx
+++ b/data/harga_emas_antam.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Metadata" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Harga Emas'!$A$1:$D$5044</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Harga Emas'!$A$1:$D$5047</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5044"/>
+  <dimension ref="A1:D5047"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -65101,8 +65101,50 @@
         <v>150000</v>
       </c>
     </row>
+    <row r="5045">
+      <c r="A5045" s="2" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B5045" s="3" t="n">
+        <v>2604000</v>
+      </c>
+      <c r="C5045" s="3" t="n">
+        <v>2454000</v>
+      </c>
+      <c r="D5045" s="3" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="5046">
+      <c r="A5046" s="2" t="n">
+        <v>46279</v>
+      </c>
+      <c r="B5046" s="3" t="n">
+        <v>2602000</v>
+      </c>
+      <c r="C5046" s="3" t="n">
+        <v>2452000</v>
+      </c>
+      <c r="D5046" s="3" t="n">
+        <v>150000</v>
+      </c>
+    </row>
+    <row r="5047">
+      <c r="A5047" s="2" t="n">
+        <v>46280</v>
+      </c>
+      <c r="B5047" s="3" t="n">
+        <v>2592000</v>
+      </c>
+      <c r="C5047" s="3" t="n">
+        <v>2437000</v>
+      </c>
+      <c r="D5047" s="3" t="n">
+        <v>155000</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D5044"/>
+  <autoFilter ref="A1:D5047"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -65152,7 +65194,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-09-12 14:16:29 WIB</t>
+          <t>2026-09-15 14:56:05 WIB</t>
         </is>
       </c>
     </row>
@@ -65163,7 +65205,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>5043</v>
+        <v>5046</v>
       </c>
     </row>
   </sheetData>

</xml_diff>